<commit_message>
Fix use-case diagram layout/relationships and correct NFR-001 in requirements table
</commit_message>
<xml_diff>
--- a/Lab-1/Requirements_Table_Pharmacy_Expiry_Reorder.xlsx
+++ b/Lab-1/Requirements_Table_Pharmacy_Expiry_Reorder.xlsx
@@ -658,7 +658,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>The system shall automatically generate and dispatch supplier purchase order requests when item stock dips below safety threshold.</t>
+          <t>The system shall transmit purchase order requests to suppliers over an authenticated, encrypted channel and confirm successful delivery within 5 seconds of generation.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -668,12 +668,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Pass: benchmarking tests confirm target latency and security standards under simulated peak load.</t>
+          <t>Pass: 95% of purchase order requests are delivered over a TLS-encrypted, authenticated connection with delivery confirmation received within 5 seconds, under simulated peak load. Fail: any request is sent unencrypted, unauthenticated, or confirmation exceeds 5 seconds.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Ensures replenishment actions occur automatically and reliably under operational load.</t>
+          <t>Protects sensitive supplier and stock data in transit and ensures replenishment orders are dispatched reliably without delay, distinct from the functional trigger already captured in FR-005.</t>
         </is>
       </c>
     </row>

</xml_diff>